<commit_message>
docs: CON-01 사용 여부 저장 위치를 status_code로 한정
사용 여부 저장 위치에서 BS_SERVICE.active_yn 제외, BS_SERVICE_VERSION.
status_code만 유지. active_yn은 최초 등록 시 Y 고정·미변경. (별첨D v1.3)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨D_화면설계서.xlsx
+++ b/docs/별첨D_화면설계서.xlsx
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -697,6 +697,33 @@
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>테이블설계서 대조 시 누락 확인 — BS_SERVICE.service_type NOT NULL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>v1.3</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>DBInc</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>CON-01 사용 여부 저장 위치를 BS_SERVICE_VERSION.status_code로 한정</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>bs_service.active_yn은 최초 등록 시 Y 고정·미변경</t>
         </is>
       </c>
     </row>
@@ -1518,12 +1545,12 @@
       </c>
       <c r="D25" s="11" t="inlineStr">
         <is>
-          <t>BS_SERVICE.active_yn + BS_SERVICE_VERSION.status_code</t>
+          <t>BS_SERVICE_VERSION.status_code</t>
         </is>
       </c>
       <c r="E25" s="11" t="inlineStr">
         <is>
-          <t>사용→active_yn=Y &amp; status_code=ACTIVE / 미사용→N &amp; INACTIVE · '사용' 저장 시 Bean 재검증</t>
+          <t>사용→ACTIVE / 미사용→INACTIVE · '사용' 저장 시 Bean 재검증 (bs_service.active_yn은 최초 등록 시 Y 고정, 미변경)</t>
         </is>
       </c>
       <c r="F25" s="11" t="inlineStr">

</xml_diff>

<commit_message>
docs: CON-01 저장 버튼 처리 설명 보강 (버전 확인 후 UPDATE/INSERT)
저장 시 버전 변경 처리 명시: 해당 버전이 있으면 UPDATE, 없으면 신규
버전 INSERT. (별첨D v1.4)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLMxyQgKYFz74Rk29M4m6g
</commit_message>
<xml_diff>
--- a/docs/별첨D_화면설계서.xlsx
+++ b/docs/별첨D_화면설계서.xlsx
@@ -576,7 +576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -726,6 +726,29 @@
           <t>bs_service.active_yn은 최초 등록 시 Y 고정·미변경</t>
         </is>
       </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>v1.4</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>DBInc</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>CON-01 저장 처리 설명 보강(버전 확인 후 UPDATE/INSERT)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1651,7 +1674,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Bean 존재·Interface 구현·Service ID/버전 일치 검증 후 저장. 사용=저장 시 Registry 갱신→외부 호출 허용</t>
+          <t>Bean·Interface·Service ID 검증 후 저장. 버전 변경 시: 해당 버전이 있으면 UPDATE, 없으면 신규 버전 INSERT. 사용=저장 시 Registry 갱신→외부 호출 허용</t>
         </is>
       </c>
     </row>

</xml_diff>